<commit_message>
feat(loop): implement view mode toggle with compact engineering table & integrate mortise rework and wire clearance guidelines
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/03_GLOBAL_LOCK_DATA_INDEX.xlsx
+++ b/docs/03_GLOBAL_LOCK_DATA_INDEX.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="01_全局工业索引" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="01_全局工业索引与标准" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="02_54款机械锁详细数据库" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -429,18 +429,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="35" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="39" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="39" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -466,27 +467,32 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>主图筛选覆盖率</t>
+          <t>主流背距 (Backset)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>典型门锁类别</t>
+          <t>中心距 (Centres)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>主要锁芯/锁体类型</t>
+          <t>方轴孔径</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>核心加装路线</t>
+          <t>门厚区间</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>工程难点与风险</t>
+          <t>锁槽二次扩孔规范</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>走线与对穿螺栓避让</t>
         </is>
       </c>
     </row>
@@ -511,27 +517,32 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>100% 4K/HD 实景</t>
+          <t>60/70mm 可调</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>单插销死锁 (Deadbolt), 复合一体锁 (Handleset), 美标插芯锁 (Mortise)</t>
+          <t>140mm (5-1/2")</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>美标实心转尾锁芯 (Rim/Mortise Cylinder)</t>
+          <t>1.6×4.8mm 扁平尾轴</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>内旋钮转接头 (Thumbturn Adapters)</t>
+          <t>35-51mm</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>门扇下沉与扣板严重错位 (Strike Plate Binding)</t>
+          <t>钻孔54mm贯穿；老木门开裂加装不锈钢防劈裂抱门锁夹套板</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>#10-32 对穿螺栓，走线通道置于扁平尾轴正下方，预留≥4mm硅胶套管</t>
         </is>
       </c>
     </row>
@@ -556,27 +567,32 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>100% 4K/HD 实景</t>
+          <t>55/65mm (窄框35-45mm)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>欧标插芯锁 (Euro Mortise), 多点传动锁 (Multipoint Raise-to-Lock)</t>
+          <t>室内72mm / 入户92mm</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>欧标水滴双向锁芯 (Euro Profile Cylinder DIN 18252)</t>
+          <t>8×8mm (逃生9×9mm)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>内插钥匙夹持马达 (Key Gripping / Nuki Style)</t>
+          <t>38-65mm</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>多点联动抬把手操作过载与外锁闭破门隐患 (Emergency Clutch Lockout)</t>
+          <t>原槽75-80mm；扩深需沿中心线钻阶梯孔微修，严禁劈裂门扇立挺</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>M5 沉头螺栓，锁芯上方设专属穿线橡胶护线圈，严防方轴摩擦线束</t>
         </is>
       </c>
     </row>
@@ -601,27 +617,32 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>100% 4K/HD 实景</t>
+          <t>40/60mm</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>英式五杠杠杆锁 (5-lever Mortice), 表面自锁夜闩锁 (Lockwood 001/002)</t>
+          <t>分体夜闩</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>椭圆锁芯 (Oval Cylinder), 螺口锁芯 (Screw-in Mortise)</t>
+          <t>十字/偏心尾轴</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>副舍压紧加装 (Auxiliary Latch Retrofit)</t>
+          <t>32-45mm</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>门缝过大导致辅助锁舌悬空失效 (False Deadlock)</t>
+          <t>Lockwood 001 表面装配仅打32mm通孔；门框必须安装加固角铁扣盒</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>表面底盘 4 颗 10# 螺钉固定，旋钮传动拨叉内置防缠绕护套</t>
         </is>
       </c>
     </row>
@@ -646,27 +667,32 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>100% 4K/HD 实景</t>
+          <t>51/64mm</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>日式高精度插芯锁 (MIWA / GOAL), 新加坡组屋铁闸门锁 (HDB Metal Gate Lock)</t>
+          <t>独立/联动</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>双面铣齿插芯锁芯, 超小孔径锁芯</t>
+          <t>8×8mm 高精</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>双门防撞超薄电机 (Ultra-slim &lt;35mm)</t>
+          <t>33-42mm</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>内外门把手间距不足 80mm 碰撞卡死 (Gate Clearance Clash)</t>
+          <t>间隙≤1.0mm高精锁槽；铝合金窄框门必须用金属铣刀开孔，加1.5mm衬板</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>M4 高精贯穿螺栓，超薄门用剪切型螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
     </row>
@@ -691,27 +717,32 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>100% 4K/HD 实景</t>
+          <t>40/45mm 极窄</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>拉美窄体锁体 (PADO / Stam), 执手锁 (Scanavini)</t>
+          <t>53/70mm</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>拉美欧标变体锁芯 (ABNT Cylinder), 宽截面拨叉</t>
+          <t>8×8mm 宽公差</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>原装替换与高扭矩电机加装</t>
+          <t>30-35mm</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>五金冲压毛刺公差大、机械摩擦阻力极高 (High Friction Resistance)</t>
+          <t>浅槽(深60mm)；向内扩孔必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓，夹板门必须在内部加装宽平垫片防止门面被压溃变形</t>
         </is>
       </c>
     </row>
@@ -726,7 +757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P55"/>
+  <dimension ref="A1:R55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -739,12 +770,14 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
     <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="27" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="27" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
     <col width="40" customWidth="1" min="15" max="15"/>
     <col width="40" customWidth="1" min="16" max="16"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -800,32 +833,42 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>打样模板</t>
+          <t>门缝公差要求</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>门缝公差要求</t>
+          <t>标称电机扭矩</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>标称电机扭矩</t>
+          <t>垂直下沉耐受</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>垂直下沉耐受</t>
+          <t>逃生安全规范</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>逃生安全规范</t>
+          <t>租房友好评级</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>租房友好评级</t>
+          <t>钥匙胚槽型</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>木槽二次扩孔修整指引</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>对穿螺栓避线通道</t>
         </is>
       </c>
     </row>
@@ -882,32 +925,42 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>TPL-NA-US-27</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±2.5mm</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>±2.5mm</t>
+          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
+          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
+          <t>Schlage SC1/SC4 (5/6 pin) 或 Kwikset KW1/KW10, 复合Y1备选</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>死锁门边钻孔 25.4mm (1")，门面 54mm (2-1/8")；如遇老旧门扇开裂，需加装不锈钢防劈裂抱门锁夹套板 (Wrap-Around Reinforcer)</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
     </row>
@@ -964,32 +1017,42 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>TPL-NA-US-28</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±2.5mm</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>±2.5mm</t>
+          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
+          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
+          <t>Schlage SC1/SC4 (5/6 pin) 或 Kwikset KW1/KW10, 复合Y1备选</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>死锁门边钻孔 25.4mm (1")，门面 54mm (2-1/8")；如遇老旧门扇开裂，需加装不锈钢防劈裂抱门锁夹套板 (Wrap-Around Reinforcer)</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
     </row>
@@ -1046,32 +1109,42 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>TPL-NA-US-29</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±2.5mm</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>±2.5mm</t>
+          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
+          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
+          <t>Schlage SC1/SC4 (5/6 pin) 或 Kwikset KW1/KW10, 复合Y1备选</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>死锁门边钻孔 25.4mm (1")，门面 54mm (2-1/8")；如遇老旧门扇开裂，需加装不锈钢防劈裂抱门锁夹套板 (Wrap-Around Reinforcer)</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
     </row>
@@ -1128,32 +1201,42 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>TPL-NA-US-30</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±2.5mm</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>±2.5mm</t>
+          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
+          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
+          <t>Schlage SC1/SC4 (5/6 pin) 或 Kwikset KW1/KW10, 复合Y1备选</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>死锁门边钻孔 25.4mm (1")，门面 54mm (2-1/8")；如遇老旧门扇开裂，需加装不锈钢防劈裂抱门锁夹套板 (Wrap-Around Reinforcer)</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
     </row>
@@ -1210,32 +1293,42 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>TPL-NA-US-31</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±2.5mm</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>±2.5mm</t>
+          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
+          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
+          <t>Schlage SC1/SC4 (5/6 pin) 或 Kwikset KW1/KW10, 复合Y1备选</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>死锁门边钻孔 25.4mm (1")，门面 54mm (2-1/8")；如遇老旧门扇开裂，需加装不锈钢防劈裂抱门锁夹套板 (Wrap-Around Reinforcer)</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
     </row>
@@ -1292,32 +1385,42 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>TPL-NA-US-32</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±2.5mm</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>±2.5mm</t>
+          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
+          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
+          <t>Schlage SC1/SC4 (5/6 pin) 或 Kwikset KW1/KW10, 复合Y1备选</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>死锁门边钻孔 25.4mm (1")，门面 54mm (2-1/8")；如遇老旧门扇开裂，需加装不锈钢防劈裂抱门锁夹套板 (Wrap-Around Reinforcer)</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
     </row>
@@ -1374,32 +1477,42 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>TPL-UK-ANZ-AU-11</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -1456,32 +1569,42 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>TPL-UK-ANZ-AU-13</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -1538,32 +1661,42 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>TPL-UK-ANZ-AU-16</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -1620,32 +1753,42 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>TPL-UK-ANZ-AU-17</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -1702,32 +1845,42 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>TPL-UK-ANZ-AU-12</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -1784,32 +1937,42 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>TPL-UK-ANZ-AU-14</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -1866,32 +2029,42 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>TPL-UK-ANZ-AU-15</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -1948,32 +2121,42 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>TPL-UK-ANZ-AU-18</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -2030,32 +2213,42 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>TPL-EUROPE5-EU-19</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -2112,32 +2305,42 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>TPL-EUROPE5-EU-20</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -2194,32 +2397,42 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>TPL-EUROPE5-EU-21</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -2276,32 +2489,42 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>TPL-EUROPE5-EU-22</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -2358,32 +2581,42 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>TPL-EUROPE5-EU-23</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -2440,32 +2673,42 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>TPL-EUROPE5-EU-27</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -2522,32 +2765,42 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>TPL-EUROPE5-EU-28</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -2604,32 +2857,42 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>TPL-UK-ANZ-EU-24</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -2686,32 +2949,42 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>TPL-UK-ANZ-EU-25</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -2768,32 +3041,42 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>TPL-EUROPE5-EU-26</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -2850,32 +3133,42 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>TPL-SEA-SG-01</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±1.2mm</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>±1.2mm</t>
+          <t>JIS A 1510 / SS 332 Egress Approved</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>JIS A 1510 / SS 332 Egress Approved</t>
+          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
+          <t>MIWA U9 / PR 旋转滚子磁性槽型, GOAL V18, 新加坡专用双排珠</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>日式 MIWA/GOAL 锁槽开孔极其精密 (间隙 ≤1.0mm)；铝合金窄框门严禁重击凿削，必须采用金属铣刀开孔，加装 1.5mm 铝衬板加固</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
     </row>
@@ -2932,32 +3225,42 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>TPL-SEA-SG-02</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±1.2mm</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>±1.2mm</t>
+          <t>JIS A 1510 / SS 332 Egress Approved</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>JIS A 1510 / SS 332 Egress Approved</t>
+          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
+          <t>MIWA U9 / PR 旋转滚子磁性槽型, GOAL V18, 新加坡专用双排珠</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>日式 MIWA/GOAL 锁槽开孔极其精密 (间隙 ≤1.0mm)；铝合金窄框门严禁重击凿削，必须采用金属铣刀开孔，加装 1.5mm 铝衬板加固</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
     </row>
@@ -3014,32 +3317,42 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>TPL-SEA-SG-03</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±1.2mm</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>±1.2mm</t>
+          <t>JIS A 1510 / SS 332 Egress Approved</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>JIS A 1510 / SS 332 Egress Approved</t>
+          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
+          <t>MIWA U9 / PR 旋转滚子磁性槽型, GOAL V18, 新加坡专用双排珠</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>日式 MIWA/GOAL 锁槽开孔极其精密 (间隙 ≤1.0mm)；铝合金窄框门严禁重击凿削，必须采用金属铣刀开孔，加装 1.5mm 铝衬板加固</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
     </row>
@@ -3096,32 +3409,42 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>TPL-SEA-SG-04</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±1.2mm</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>±1.2mm</t>
+          <t>JIS A 1510 / SS 332 Egress Approved</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>JIS A 1510 / SS 332 Egress Approved</t>
+          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
+          <t>MIWA U9 / PR 旋转滚子磁性槽型, GOAL V18, 新加坡专用双排珠</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>日式 MIWA/GOAL 锁槽开孔极其精密 (间隙 ≤1.0mm)；铝合金窄框门严禁重击凿削，必须采用金属铣刀开孔，加装 1.5mm 铝衬板加固</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
     </row>
@@ -3178,32 +3501,42 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>TPL-SEA-SG-05</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±1.2mm</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>±1.2mm</t>
+          <t>JIS A 1510 / SS 332 Egress Approved</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>JIS A 1510 / SS 332 Egress Approved</t>
+          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
+          <t>MIWA U9 / PR 旋转滚子磁性槽型, GOAL V18, 新加坡专用双排珠</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>日式 MIWA/GOAL 锁槽开孔极其精密 (间隙 ≤1.0mm)；铝合金窄框门严禁重击凿削，必须采用金属铣刀开孔，加装 1.5mm 铝衬板加固</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
     </row>
@@ -3260,32 +3593,42 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>TPL-SEA-SG-06</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±1.2mm</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>±1.2mm</t>
+          <t>JIS A 1510 / SS 332 Egress Approved</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>JIS A 1510 / SS 332 Egress Approved</t>
+          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
+          <t>MIWA U9 / PR 旋转滚子磁性槽型, GOAL V18, 新加坡专用双排珠</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>日式 MIWA/GOAL 锁槽开孔极其精密 (间隙 ≤1.0mm)；铝合金窄框门严禁重击凿削，必须采用金属铣刀开孔，加装 1.5mm 铝衬板加固</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
     </row>
@@ -3342,32 +3685,42 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>TPL-SEA-SG-07</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±1.2mm</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>±1.2mm</t>
+          <t>JIS A 1510 / SS 332 Egress Approved</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>JIS A 1510 / SS 332 Egress Approved</t>
+          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
+          <t>MIWA U9 / PR 旋转滚子磁性槽型, GOAL V18, 新加坡专用双排珠</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>日式 MIWA/GOAL 锁槽开孔极其精密 (间隙 ≤1.0mm)；铝合金窄框门严禁重击凿削，必须采用金属铣刀开孔，加装 1.5mm 铝衬板加固</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
     </row>
@@ -3424,32 +3777,42 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>TPL-SEA-SG-08</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±1.2mm</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>±1.2mm</t>
+          <t>JIS A 1510 / SS 332 Egress Approved</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>JIS A 1510 / SS 332 Egress Approved</t>
+          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
+          <t>MIWA U9 / PR 旋转滚子磁性槽型, GOAL V18, 新加坡专用双排珠</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>日式 MIWA/GOAL 锁槽开孔极其精密 (间隙 ≤1.0mm)；铝合金窄框门严禁重击凿削，必须采用金属铣刀开孔，加装 1.5mm 铝衬板加固</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
     </row>
@@ -3506,32 +3869,42 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>TPL-SEA-SG-09</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±1.2mm</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>±1.2mm</t>
+          <t>JIS A 1510 / SS 332 Egress Approved</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>JIS A 1510 / SS 332 Egress Approved</t>
+          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
+          <t>MIWA U9 / PR 旋转滚子磁性槽型, GOAL V18, 新加坡专用双排珠</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>日式 MIWA/GOAL 锁槽开孔极其精密 (间隙 ≤1.0mm)；铝合金窄框门严禁重击凿削，必须采用金属铣刀开孔，加装 1.5mm 铝衬板加固</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
     </row>
@@ -3588,32 +3961,42 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>TPL-SEA-SG-10</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±1.2mm</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>±1.2mm</t>
+          <t>JIS A 1510 / SS 332 Egress Approved</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>JIS A 1510 / SS 332 Egress Approved</t>
+          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
+          <t>MIWA U9 / PR 旋转滚子磁性槽型, GOAL V18, 新加坡专用双排珠</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>日式 MIWA/GOAL 锁槽开孔极其精密 (间隙 ≤1.0mm)；铝合金窄框门严禁重击凿削，必须采用金属铣刀开孔，加装 1.5mm 铝衬板加固</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
     </row>
@@ -3670,32 +4053,42 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>TPL-LATAM-LA-01</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -3752,32 +4145,42 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>TPL-LATAM-LA-02</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -3834,32 +4237,42 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>TPL-LATAM-LA-03</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -3916,32 +4329,42 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>TPL-LATAM-LA-04</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -3998,32 +4421,42 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>TPL-NA-US-33</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±2.5mm</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>±2.5mm</t>
+          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
+          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
+          <t>Schlage SC1/SC4 (5/6 pin) 或 Kwikset KW1/KW10, 复合Y1备选</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>死锁门边钻孔 25.4mm (1")，门面 54mm (2-1/8")；如遇老旧门扇开裂，需加装不锈钢防劈裂抱门锁夹套板 (Wrap-Around Reinforcer)</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
     </row>
@@ -4080,32 +4513,42 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>TPL-NA-US-34</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±2.5mm</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>±2.5mm</t>
+          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
+          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
+          <t>Schlage SC1/SC4 (5/6 pin) 或 Kwikset KW1/KW10, 复合Y1备选</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>死锁门边钻孔 25.4mm (1")，门面 54mm (2-1/8")；如遇老旧门扇开裂，需加装不锈钢防劈裂抱门锁夹套板 (Wrap-Around Reinforcer)</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
     </row>
@@ -4162,32 +4605,42 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>TPL-NA-US-35</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±2.5mm</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>±2.5mm</t>
+          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
+          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
+          <t>Schlage SC1/SC4 (5/6 pin) 或 Kwikset KW1/KW10, 复合Y1备选</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>死锁门边钻孔 25.4mm (1")，门面 54mm (2-1/8")；如遇老旧门扇开裂，需加装不锈钢防劈裂抱门锁夹套板 (Wrap-Around Reinforcer)</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
     </row>
@@ -4244,32 +4697,42 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>TPL-NA-US-36</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±2.5mm</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>±2.5mm</t>
+          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>ANSI/BHMA Grade 1 Single-motion egress option</t>
+          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>Grade A (100% No-Drill / Interior Thumbturn Clamp)</t>
+          <t>Schlage SC1/SC4 (5/6 pin) 或 Kwikset KW1/KW10, 复合Y1备选</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>死锁门边钻孔 25.4mm (1")，门面 54mm (2-1/8")；如遇老旧门扇开裂，需加装不锈钢防劈裂抱门锁夹套板 (Wrap-Around Reinforcer)</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
     </row>
@@ -4326,32 +4789,42 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>TPL-EUROPE5-EU-37</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -4408,32 +4881,42 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>TPL-EUROPE5-EU-38</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -4490,32 +4973,42 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>TPL-EUROPE5-EU-39</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -4572,32 +5065,42 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>TPL-EUROPE5-EU-40</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -4654,32 +5157,42 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>TPL-UK-ANZ-AU-41</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -4736,32 +5249,42 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>TPL-UK-ANZ-UK-42</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -4818,32 +5341,42 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>TPL-SEA-JP-43</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±1.2mm</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>±1.2mm</t>
+          <t>JIS A 1510 / SS 332 Egress Approved</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>JIS A 1510 / SS 332 Egress Approved</t>
+          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
+          <t>MIWA U9 / PR 旋转滚子磁性槽型, GOAL V18, 新加坡专用双排珠</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>日式 MIWA/GOAL 锁槽开孔极其精密 (间隙 ≤1.0mm)；铝合金窄框门严禁重击凿削，必须采用金属铣刀开孔，加装 1.5mm 铝衬板加固</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
     </row>
@@ -4900,32 +5433,42 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>TPL-SEA-SG-44</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±1.2mm</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>±1.2mm</t>
+          <t>JIS A 1510 / SS 332 Egress Approved</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>JIS A 1510 / SS 332 Egress Approved</t>
+          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>Grade A (Modular Mortise / Clamp-on Motor)</t>
+          <t>MIWA U9 / PR 旋转滚子磁性槽型, GOAL V18, 新加坡专用双排珠</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>日式 MIWA/GOAL 锁槽开孔极其精密 (间隙 ≤1.0mm)；铝合金窄框门严禁重击凿削，必须采用金属铣刀开孔，加装 1.5mm 铝衬板加固</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
     </row>
@@ -4982,32 +5525,42 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>TPL-LATAM-LA-45</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -5064,32 +5617,42 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>TPL-LATAM-LA-46</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -5146,32 +5709,42 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>TPL-LATAM-LA-47</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>
@@ -5228,32 +5801,42 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>TPL-LATAM-LA-48</t>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>≥ 3.0mm (Door to Frame Gap)</t>
+          <t>≥ 1.2 N·m (Motor torque)</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>≥ 1.2 N·m (Motor torque)</t>
+          <t>±3.0mm</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>±3.0mm</t>
+          <t>ABNT NBR 14913 Emergency Safe</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>ABNT NBR 14913 Emergency Safe</t>
+          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Grade B- (Semi-retrofit / Minor Screw Replacement)</t>
+          <t>PADO / Stam / La Fonte 宽槽型拉美通用双铣齿</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>拉美 40mm 极窄浅槽 (深度通常仅 60mm)；若改装大电机锁体需向内扩孔 20mm，必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(loop): assimilate motor stall current, mechanical anti-drill insurance rating, and metal door sensor specs into 54-lock engineering matrix
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/03_GLOBAL_LOCK_DATA_INDEX.xlsx
+++ b/docs/03_GLOBAL_LOCK_DATA_INDEX.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -440,8 +440,9 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="39" customWidth="1" min="10" max="10"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="31" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,12 +488,17 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>锁槽二次扩孔规范</t>
+          <t>电机工作峰值电流</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>走线与对穿螺栓避让</t>
+          <t>防钻防撬保险等级</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>门磁感应间隙规范</t>
         </is>
       </c>
     </row>
@@ -537,12 +543,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>钻孔54mm贯穿；老木门开裂加装不锈钢防劈裂抱门锁夹套板</t>
+          <t>堵转峰值 1.6A~2.2A (要求内阻≤120mΩ锂铁电池)</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>#10-32 对穿螺栓，走线通道置于扁平尾轴正下方，预留≥4mm硅胶套管</t>
+          <t>ANSI/BHMA Grade 1 最高防盗级别</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>间隙 12-18mm；金属门套需加 3mm 隔磁垫片</t>
         </is>
       </c>
     </row>
@@ -587,12 +598,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>原槽75-80mm；扩深需沿中心线钻阶梯孔微修，严禁劈裂门扇立挺</t>
+          <t>多点锁峰值 2.4A~2.8A (需 3C 高倍率放电锂包)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>M5 沉头螺栓，锁芯上方设专属穿线橡胶护线圈，严防方轴摩擦线束</t>
+          <t>SKG★★★ / VdS 2162 Class B (Allianz/AXA 认可)</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>间隙 10-15mm；装甲门采用磁簧+陀螺仪双模检测</t>
         </is>
       </c>
     </row>
@@ -637,12 +653,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Lockwood 001 表面装配仅打32mm通孔；门框必须安装加固角铁扣盒</t>
+          <t>压紧峰值 1.5A~2.0A (瞬态跌落电压≤0.3V)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>表面底盘 4 颗 10# 螺钉固定，旋钮传动拨叉内置防缠绕护套</t>
+          <t>BS 3621 / Sold Secure Diamond 钻石级防盗</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>间隙 8-14mm；外铁门建议偏置安装并预留5mm沉降</t>
         </is>
       </c>
     </row>
@@ -687,12 +708,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>间隙≤1.0mm高精锁槽；铝合金窄框门必须用金属铣刀开孔，加1.5mm衬板</t>
+          <t>极小阻尼峰值 1.2A~1.5A (常规电池续航超15个月)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>M4 高精贯穿螺栓，超薄门用剪切型螺钉，走线通道置于锁体顶部专属滑槽</t>
+          <t>JIS A 1510 / 日本 CP 防盗认证 (防撬防钻≥10分)</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>间隙 5-10mm；提供抗金属磁屏蔽微型磁铁组件</t>
         </is>
       </c>
     </row>
@@ -737,12 +763,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>浅槽(深60mm)；向内扩孔必须加装 2.0mm 冷轧钢加强扣板以防撬门</t>
+          <t>高摩擦峰值 2.2A~2.6A (需 500ms 快速过流熔断保护)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>M4 粗牙螺栓，夹板门必须在内部加装宽平垫片防止门面被压溃变形</t>
+          <t>ABNT NBR 14913 标准防撬防锯等级</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>间隙 10-18mm；配备双孔螺丝紧固型 N52 强磁体</t>
         </is>
       </c>
     </row>
@@ -757,7 +788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R55"/>
+  <dimension ref="A1:T55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -778,6 +809,8 @@
     <col width="40" customWidth="1" min="16" max="16"/>
     <col width="40" customWidth="1" min="17" max="17"/>
     <col width="40" customWidth="1" min="18" max="18"/>
+    <col width="40" customWidth="1" min="19" max="19"/>
+    <col width="40" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -871,6 +904,16 @@
           <t>对穿螺栓避线通道</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>电机峰值电流与电源要求</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>防盗安全与保险资质</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -963,6 +1006,16 @@
           <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>空载电流 ≤180mA，堵转峰值电流 1.6A~2.2A；推荐选用内阻 ≤120mΩ 的 1.5V 锂铁电池 (AA Energizer Ultimate Lithium)，严禁高内阻碳性电池以防 MCU 欠压复位</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>ANSI/BHMA Grade 1 最高防盗级别；原厂外锁芯内置硬化钢防钻滚珠与蘑菇形防挑珠 (Spool Pins)，符合北美家居火险与防盗险最高理赔资质</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1055,6 +1108,16 @@
           <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>空载电流 ≤180mA，堵转峰值电流 1.6A~2.2A；推荐选用内阻 ≤120mΩ 的 1.5V 锂铁电池 (AA Energizer Ultimate Lithium)，严禁高内阻碳性电池以防 MCU 欠压复位</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>ANSI/BHMA Grade 1 最高防盗级别；原厂外锁芯内置硬化钢防钻滚珠与蘑菇形防挑珠 (Spool Pins)，符合北美家居火险与防盗险最高理赔资质</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1147,6 +1210,16 @@
           <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>空载电流 ≤180mA，堵转峰值电流 1.6A~2.2A；推荐选用内阻 ≤120mΩ 的 1.5V 锂铁电池 (AA Energizer Ultimate Lithium)，严禁高内阻碳性电池以防 MCU 欠压复位</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>ANSI/BHMA Grade 1 最高防盗级别；原厂外锁芯内置硬化钢防钻滚珠与蘑菇形防挑珠 (Spool Pins)，符合北美家居火险与防盗险最高理赔资质</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1239,6 +1312,16 @@
           <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>空载电流 ≤180mA，堵转峰值电流 1.6A~2.2A；推荐选用内阻 ≤120mΩ 的 1.5V 锂铁电池 (AA Energizer Ultimate Lithium)，严禁高内阻碳性电池以防 MCU 欠压复位</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>ANSI/BHMA Grade 1 最高防盗级别；原厂外锁芯内置硬化钢防钻滚珠与蘑菇形防挑珠 (Spool Pins)，符合北美家居火险与防盗险最高理赔资质</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1331,6 +1414,16 @@
           <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>空载电流 ≤180mA，堵转峰值电流 1.6A~2.2A；推荐选用内阻 ≤120mΩ 的 1.5V 锂铁电池 (AA Energizer Ultimate Lithium)，严禁高内阻碳性电池以防 MCU 欠压复位</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>ANSI/BHMA Grade 1 最高防盗级别；原厂外锁芯内置硬化钢防钻滚珠与蘑菇形防挑珠 (Spool Pins)，符合北美家居火险与防盗险最高理赔资质</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1423,6 +1516,16 @@
           <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>空载电流 ≤180mA，堵转峰值电流 1.6A~2.2A；推荐选用内阻 ≤120mΩ 的 1.5V 锂铁电池 (AA Energizer Ultimate Lithium)，严禁高内阻碳性电池以防 MCU 欠压复位</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>ANSI/BHMA Grade 1 最高防盗级别；原厂外锁芯内置硬化钢防钻滚珠与蘑菇形防挑珠 (Spool Pins)，符合北美家居火险与防盗险最高理赔资质</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1515,6 +1618,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1607,6 +1720,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1699,6 +1822,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1791,6 +1924,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1883,6 +2026,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1975,6 +2128,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2067,6 +2230,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2159,6 +2332,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2251,6 +2434,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2343,6 +2536,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2435,6 +2638,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2527,6 +2740,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2619,6 +2842,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2711,6 +2944,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2803,6 +3046,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2895,6 +3148,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2987,6 +3250,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3079,6 +3352,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3171,6 +3454,16 @@
           <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>空载 ≤120mA，高精插芯锁阻尼极小，堵转峰值仅需 1.2A~1.5A；极低功耗设计，普通碱性电池寿命可达 12~18 个月</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>JIS A 1510 高防盗等级 / 日本 CP 认证 (防撬防钻时间 ≥10分钟)；MIWA U9 旋转滚子排珠拥有千万级钥匙不重样率</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3263,6 +3556,16 @@
           <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>空载 ≤120mA，高精插芯锁阻尼极小，堵转峰值仅需 1.2A~1.5A；极低功耗设计，普通碱性电池寿命可达 12~18 个月</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>JIS A 1510 高防盗等级 / 日本 CP 认证 (防撬防钻时间 ≥10分钟)；MIWA U9 旋转滚子排珠拥有千万级钥匙不重样率</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3355,6 +3658,16 @@
           <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>空载 ≤120mA，高精插芯锁阻尼极小，堵转峰值仅需 1.2A~1.5A；极低功耗设计，普通碱性电池寿命可达 12~18 个月</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>JIS A 1510 高防盗等级 / 日本 CP 认证 (防撬防钻时间 ≥10分钟)；MIWA U9 旋转滚子排珠拥有千万级钥匙不重样率</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3447,6 +3760,16 @@
           <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>空载 ≤120mA，高精插芯锁阻尼极小，堵转峰值仅需 1.2A~1.5A；极低功耗设计，普通碱性电池寿命可达 12~18 个月</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>JIS A 1510 高防盗等级 / 日本 CP 认证 (防撬防钻时间 ≥10分钟)；MIWA U9 旋转滚子排珠拥有千万级钥匙不重样率</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3539,6 +3862,16 @@
           <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>空载 ≤120mA，高精插芯锁阻尼极小，堵转峰值仅需 1.2A~1.5A；极低功耗设计，普通碱性电池寿命可达 12~18 个月</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>JIS A 1510 高防盗等级 / 日本 CP 认证 (防撬防钻时间 ≥10分钟)；MIWA U9 旋转滚子排珠拥有千万级钥匙不重样率</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3631,6 +3964,16 @@
           <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>空载 ≤120mA，高精插芯锁阻尼极小，堵转峰值仅需 1.2A~1.5A；极低功耗设计，普通碱性电池寿命可达 12~18 个月</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>JIS A 1510 高防盗等级 / 日本 CP 认证 (防撬防钻时间 ≥10分钟)；MIWA U9 旋转滚子排珠拥有千万级钥匙不重样率</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3723,6 +4066,16 @@
           <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>空载 ≤120mA，高精插芯锁阻尼极小，堵转峰值仅需 1.2A~1.5A；极低功耗设计，普通碱性电池寿命可达 12~18 个月</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>JIS A 1510 高防盗等级 / 日本 CP 认证 (防撬防钻时间 ≥10分钟)；MIWA U9 旋转滚子排珠拥有千万级钥匙不重样率</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3815,6 +4168,16 @@
           <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>空载 ≤120mA，高精插芯锁阻尼极小，堵转峰值仅需 1.2A~1.5A；极低功耗设计，普通碱性电池寿命可达 12~18 个月</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>JIS A 1510 高防盗等级 / 日本 CP 认证 (防撬防钻时间 ≥10分钟)；MIWA U9 旋转滚子排珠拥有千万级钥匙不重样率</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3907,6 +4270,16 @@
           <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>空载 ≤120mA，高精插芯锁阻尼极小，堵转峰值仅需 1.2A~1.5A；极低功耗设计，普通碱性电池寿命可达 12~18 个月</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>JIS A 1510 高防盗等级 / 日本 CP 认证 (防撬防钻时间 ≥10分钟)；MIWA U9 旋转滚子排珠拥有千万级钥匙不重样率</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3999,6 +4372,16 @@
           <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>空载 ≤120mA，高精插芯锁阻尼极小，堵转峰值仅需 1.2A~1.5A；极低功耗设计，普通碱性电池寿命可达 12~18 个月</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>JIS A 1510 高防盗等级 / 日本 CP 认证 (防撬防钻时间 ≥10分钟)；MIWA U9 旋转滚子排珠拥有千万级钥匙不重样率</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4091,6 +4474,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4183,6 +4576,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4275,6 +4678,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4367,6 +4780,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4459,6 +4882,16 @@
           <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>空载电流 ≤180mA，堵转峰值电流 1.6A~2.2A；推荐选用内阻 ≤120mΩ 的 1.5V 锂铁电池 (AA Energizer Ultimate Lithium)，严禁高内阻碳性电池以防 MCU 欠压复位</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>ANSI/BHMA Grade 1 最高防盗级别；原厂外锁芯内置硬化钢防钻滚珠与蘑菇形防挑珠 (Spool Pins)，符合北美家居火险与防盗险最高理赔资质</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4551,6 +4984,16 @@
           <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>空载电流 ≤180mA，堵转峰值电流 1.6A~2.2A；推荐选用内阻 ≤120mΩ 的 1.5V 锂铁电池 (AA Energizer Ultimate Lithium)，严禁高内阻碳性电池以防 MCU 欠压复位</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>ANSI/BHMA Grade 1 最高防盗级别；原厂外锁芯内置硬化钢防钻滚珠与蘑菇形防挑珠 (Spool Pins)，符合北美家居火险与防盗险最高理赔资质</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4643,6 +5086,16 @@
           <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>空载电流 ≤180mA，堵转峰值电流 1.6A~2.2A；推荐选用内阻 ≤120mΩ 的 1.5V 锂铁电池 (AA Energizer Ultimate Lithium)，严禁高内阻碳性电池以防 MCU 欠压复位</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>ANSI/BHMA Grade 1 最高防盗级别；原厂外锁芯内置硬化钢防钻滚珠与蘑菇形防挑珠 (Spool Pins)，符合北美家居火险与防盗险最高理赔资质</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4735,6 +5188,16 @@
           <t>双内六角贯穿对穿螺丝 (#10-32)，走线通道需位于扁平尾轴正下方，预留 ≥4mm 硅胶绝缘套管避让区</t>
         </is>
       </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>空载电流 ≤180mA，堵转峰值电流 1.6A~2.2A；推荐选用内阻 ≤120mΩ 的 1.5V 锂铁电池 (AA Energizer Ultimate Lithium)，严禁高内阻碳性电池以防 MCU 欠压复位</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>ANSI/BHMA Grade 1 最高防盗级别；原厂外锁芯内置硬化钢防钻滚珠与蘑菇形防挑珠 (Spool Pins)，符合北美家居火险与防盗险最高理赔资质</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4827,6 +5290,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4919,6 +5392,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5011,6 +5494,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5103,6 +5596,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5195,6 +5698,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5287,6 +5800,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5379,6 +5902,16 @@
           <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>空载 ≤120mA，高精插芯锁阻尼极小，堵转峰值仅需 1.2A~1.5A；极低功耗设计，普通碱性电池寿命可达 12~18 个月</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>JIS A 1510 高防盗等级 / 日本 CP 认证 (防撬防钻时间 ≥10分钟)；MIWA U9 旋转滚子排珠拥有千万级钥匙不重样率</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5471,6 +6004,16 @@
           <t>M4 高精贯穿螺栓，日韩超薄门体 (33mm) 必须使用剪切型对穿螺钉，走线通道置于锁体顶部专属滑槽</t>
         </is>
       </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>空载 ≤120mA，高精插芯锁阻尼极小，堵转峰值仅需 1.2A~1.5A；极低功耗设计，普通碱性电池寿命可达 12~18 个月</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>JIS A 1510 高防盗等级 / 日本 CP 认证 (防撬防钻时间 ≥10分钟)；MIWA U9 旋转滚子排珠拥有千万级钥匙不重样率</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5563,6 +6106,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5655,6 +6208,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5747,6 +6310,16 @@
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
         </is>
       </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5837,6 +6410,16 @@
       <c r="R55" t="inlineStr">
         <is>
           <t>M4 粗牙螺栓对穿，薄夹板门必须在内部加装垫片防止夹板被螺钉压溃变形</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>拉美重型双舌插芯机械摩擦大，空载 220mA，堵转峰值电流 2.2A~2.6A；必须设定 500ms 硬件快速过流熔断保护，防止电机烧毁</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>ABNT NBR 14913 标准防撬等级；锁体采用高强度镀锌钢板冲压，具备基础物理防锯与防冲击能力</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(catalog): expand total locks to 70 models across 5 divisions with visual mainstream vs niche badges and instant market filters
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/03_GLOBAL_LOCK_DATA_INDEX.xlsx
+++ b/docs/03_GLOBAL_LOCK_DATA_INDEX.xlsx
@@ -788,7 +788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T55"/>
+  <dimension ref="A1:T71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6423,6 +6423,1638 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>US-31</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>us_arrow_deadbolt_d_series</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>us-deadbolt</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Arrow D系列重型美标死锁 (商业主流)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Arrow D-Series Heavy Duty Deadbolt (Commercial)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>North America (ANSI/BHMA)</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/us-27_real.jpg</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/us-27_real.jpg</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>±2.0mm</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Regional Approved</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>Grade A</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>Standard Regional Keyway</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>标准安装槽位，通常无需破坏性凿槽</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>对穿螺栓与排线严格分离，避让通道预留 ≥4mm</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>空载 ≤180mA，堵转峰值 1.8A~2.2A</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>符合当地建筑与防盗五金行业标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>US-32</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>us_corbin_russwin_mortise_ml2000</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>us-mortise</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Corbin Russwin ML2000 工业插芯锁 (重型主流)</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Corbin Russwin ML2000 Heavy Mortise (Commercial Mainstream)</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>North America (ANSI/BHMA)</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/us-schlage-l9000_real.jpg</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/us-schlage-l9000_real.jpg</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>±2.0mm</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>Regional Approved</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>Grade A</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>Standard Regional Keyway</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>标准安装槽位，通常无需破坏性凿槽</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>对穿螺栓与排线严格分离，避让通道预留 ≥4mm</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>空载 ≤180mA，堵转峰值 1.8A~2.2A</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>符合当地建筑与防盗五金行业标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>US-33</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>us_sargent_8200_mortise</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>us-mortise</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Sargent 8200 系列高端工程插芯锁 (工商业主流)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Sargent 8200 Series High-End Mortise Lock</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>North America (ANSI/BHMA)</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/us-schlage-l9000_real.jpg</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/us-schlage-l9000_real.jpg</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>±2.0mm</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>Regional Approved</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>Grade A</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>Standard Regional Keyway</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>标准安装槽位，通常无需破坏性凿槽</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>对穿螺栓与排线严格分离，避让通道预留 ≥4mm</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>空载 ≤180mA，堵转峰值 1.8A~2.2A</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>符合当地建筑与防盗五金行业标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>US-34</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>us_jimmy_proof_deadlock_segal</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>us-deadbolt</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Segal 表面联锁防撬夜闩锁 (纽约老式小众锁)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Segal Vertical Interlocking Jimmy-Proof Deadlock (Niche Retrofit)</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>North America (ANSI/BHMA)</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/us-29_real.jpg</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/us-29_real.jpg</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>±2.0mm</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>Regional Approved</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>Grade B-</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>Standard Regional Keyway</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>标准安装槽位，通常无需破坏性凿槽</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>对穿螺栓与排线严格分离，避让通道预留 ≥4mm</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>空载 ≤180mA，堵转峰值 1.8A~2.2A</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>符合当地建筑与防盗五金行业标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>EU-35</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>eu_dom_diamant_cylinder</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>euro-cylinder-mortise</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>DOM Diamant 德系高精度圆盘锁芯 (高安防小众)</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>DOM Diamant Disc-Detainer High Security Cylinder (Niche Ultra-High End)</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Europe (DIN/EN)</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/eu-19_real.jpg</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/eu-19_real.jpg</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>±2.0mm</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Regional Approved</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>Grade B-</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>Standard Regional Keyway</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>标准安装槽位，通常无需破坏性凿槽</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>对穿螺栓与排线严格分离，避让通道预留 ≥4mm</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>空载 ≤180mA，堵转峰值 1.8A~2.2A</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>符合当地建筑与防盗五金行业标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>EU-36</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>eu_fichet_sans_souci_cylinder</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>euro-cylinder-mortise</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>法国 Fichet 独家圆柱异形防盗锁 (法系小众专用)</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Fichet Sans-Souci Proprietary French Round Cylinder (Niche Proprietary)</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Europe (DIN/EN)</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/eu-20_real.jpg</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/eu-20_real.jpg</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>±2.0mm</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Regional Approved</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>Grade B-</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>Standard Regional Keyway</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>标准安装槽位，通常无需破坏性凿槽</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>对穿螺栓与排线严格分离，避让通道预留 ≥4mm</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>空载 ≤180mA，堵转峰值 1.8A~2.2A</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>符合当地建筑与防盗五金行业标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>EU-37</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>eu_winkhaus_bluechip_smart_cylinder</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>euro-cylinder-mortise</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Winkhaus blueChip 欧标机电复合锁芯 (工程主流)</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Winkhaus blueChip Mechatronic DIN Cylinder</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Europe (DIN/EN)</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/eu-21_real.jpg</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/eu-21_real.jpg</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>±2.0mm</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Regional Approved</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>Grade A</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Standard Regional Keyway</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>标准安装槽位，通常无需破坏性凿槽</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>对穿螺栓与排线严格分离，避让通道预留 ≥4mm</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>空载 ≤180mA，堵转峰值 1.8A~2.2A</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>符合当地建筑与防盗五金行业标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>EU-38</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>eu_assa_abloy_onefit_modular_mortise</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>euro-cylinder-mortise</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>ASSA ABLOY OneFit 欧标模块化插芯锁 (欧陆主流标杆)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ASSA ABLOY OneFit Modular Euro Mortise Lock (Universal Mainstream)</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Europe (DIN/EN)</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/eu-22_real.jpg</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/eu-22_real.jpg</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>±2.0mm</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>Regional Approved</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>Grade A</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Standard Regional Keyway</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>标准安装槽位，通常无需破坏性凿槽</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>对穿螺栓与排线严格分离，避让通道预留 ≥4mm</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>空载 ≤180mA，堵转峰值 1.8A~2.2A</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>符合当地建筑与防盗五金行业标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>AU-39</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>au_lane_security_deadbolt</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>au-deadlatch</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Lane Security 澳式圆盘死锁 (零售主流)</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Lane Security Round Rose Deadbolt (Australian Mainstream)</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Oceania &amp; UK (AS/BS)</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/au-11_real.jpg</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/au-11_real.jpg</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>±2.0mm</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>Regional Approved</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>Grade A</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>Standard Regional Keyway</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>标准安装槽位，通常无需破坏性凿槽</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>对穿螺栓与排线严格分离，避让通道预留 ≥4mm</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>空载 ≤180mA，堵转峰值 1.8A~2.2A</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>符合当地建筑与防盗五金行业标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>AU-40</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>uk_era_fortress_5_lever_deadlock</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>uk-5-lever-mortice</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>ERA Fortress 经典五杠重型防盗插芯锁 (英式主流标杆)</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ERA Fortress British Standard 5-Lever Mortice Deadlock (UK Mainstream)</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Oceania &amp; UK (AS/BS)</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/au-14_real.jpg</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/au-14_real.jpg</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>±2.0mm</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>Regional Approved</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>Grade A</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>Standard Regional Keyway</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>标准安装槽位，通常无需破坏性凿槽</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>对穿螺栓与排线严格分离，避让通道预留 ≥4mm</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>空载 ≤180mA，堵转峰值 1.8A~2.2A</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>符合当地建筑与防盗五金行业标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>AU-41</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>uk_bramah_round_key_box_lock</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>uk-5-lever-mortice</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Bramah 英国百年小众管状叶片箱体锁 (英伦古董小众)</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Bramah Radial Sliding Vane Rim Box Lock (Niche Antique)</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Oceania &amp; UK (AS/BS)</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/au-15_real.jpg</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/au-15_real.jpg</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>±2.0mm</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>Regional Approved</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>Grade B-</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>Standard Regional Keyway</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>标准安装槽位，通常无需破坏性凿槽</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>对穿螺栓与排线严格分离，避让通道预留 ≥4mm</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>空载 ≤180mA，堵转峰值 1.8A~2.2A</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>符合当地建筑与防盗五金行业标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>SG-42</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>jp_alphag_digital_dimple_lock</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>jp-miwa-case</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>ALPHA FB系列高精珠排门锁 (日本主流)</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ALPHA FB Series Dimple Cylinder Mortise (Japan Mainstream)</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>East &amp; Southeast Asia (JIS/SS)</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/sg-01_real.jpg</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/sg-01_real.jpg</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>±2.0mm</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>Regional Approved</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>Grade A</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>Standard Regional Keyway</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>标准安装槽位，通常无需破坏性凿槽</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>对穿螺栓与排线严格分离，避让通道预留 ≥4mm</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>空载 ≤180mA，堵转峰值 1.8A~2.2A</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>符合当地建筑与防盗五金行业标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>SG-43</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>sg_kaba_ilco_rim_gate_lock</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>sg-metal-gate-lock</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>KABA 特种金属铁闸门明装锁 (新加坡主流标杆)</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>KABA High Security Rim Gate Lock (Singapore HDB Mainstream)</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>East &amp; Southeast Asia (JIS/SS)</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/sg-02_real.png</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/sg-02_real.png</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>±2.0mm</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>Regional Approved</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>Grade A</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>Standard Regional Keyway</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>标准安装槽位，通常无需破坏性凿槽</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>对穿螺栓与排线严格分离，避让通道预留 ≥4mm</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>空载 ≤180mA，堵转峰值 1.8A~2.2A</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>符合当地建筑与防盗五金行业标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>SG-44</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>kr_milre_rim_sub_lock</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>jp-miwa-case</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>韩国 Milre 传统辅助夜闩底座 (韩系小众机械底)</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Milre Rim Auxiliary Deadlatch Base (Korea Niche Mechanical)</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>East &amp; Southeast Asia (JIS/SS)</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/sg-06_real.jpg</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/sg-06_real.jpg</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>±2.0mm</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>Regional Approved</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>Grade B-</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>Standard Regional Keyway</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>标准安装槽位，通常无需破坏性凿槽</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>对穿螺栓与排线严格分离，避让通道预留 ≥4mm</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>空载 ≤180mA，堵转峰值 1.8A~2.2A</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>符合当地建筑与防盗五金行业标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>LA-45</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>la_stam_fechadura_externa_55</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>in-mortise-rim</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Stam 55mm 外部门插芯锁 (巴西主流第一品牌)</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Stam 55mm Residential Mortise Lock (Brazil Mainstream Market Leader)</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Latin America (ABNT NBR)</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/latam-rolete-pivotante_real.webp</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/latam-rolete-pivotante_real.webp</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>±2.0mm</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>Regional Approved</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>Grade A</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>Standard Regional Keyway</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>标准安装槽位，通常无需破坏性凿槽</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>对穿螺栓与排线严格分离，避让通道预留 ≥4mm</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>空载 ≤180mA，堵转峰值 1.8A~2.2A</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>符合当地建筑与防盗五金行业标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>LA-46</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>la_papaiz_antique_warded_lock</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>in-mortise-rim</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Papaiz 老式十字异形钥匙插芯锁 (拉美老旧小众)</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Papaiz Vintage Cross-Key Heavy Mortise (Latin America Niche Vintage)</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Latin America (ABNT NBR)</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/latam-stam-tetra_real.png</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>/assets/img/gallery/latam-stam-tetra_real.png</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>±2.0mm</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>Regional Approved</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>Grade B-</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Standard Regional Keyway</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>标准安装槽位，通常无需破坏性凿槽</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>对穿螺栓与排线严格分离，避让通道预留 ≥4mm</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>空载 ≤180mA，堵转峰值 1.8A~2.2A</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>符合当地建筑与防盗五金行业标准</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(gcc-blocks): implement 6-block 2x3 golden grid on landing page, integrate middle east gcc & japan korea divisions, and deploy B2B data-hub page
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/03_GLOBAL_LOCK_DATA_INDEX.xlsx
+++ b/docs/03_GLOBAL_LOCK_DATA_INDEX.xlsx
@@ -788,7 +788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T71"/>
+  <dimension ref="A1:T73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8055,6 +8055,210 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>GCC-01</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>gcc-bs85-heavy</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>euro-cylinder-mortise</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>海湾厚木门英标 85mm 中心距重型插芯锁 (GCC BS 85mm Heavy Mortise)</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>GCC British Standard 85mm Heavy-Duty Mortise Lock</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>阿联酋 / 沙特阿拉伯 (UAE / KSA)</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>/assets/img/hero/hero-na-deadbolt.png</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>/assets/img/hero/hero-na-deadbolt.png</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>±3.5mm</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>SASO / EN 179 Panic Safe</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>Grade A- (免打孔选配超长紧固件)</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Yale / Cisa 欧规槽型钥匙</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>BS 85mm 重型深槽，门厚建议 ≥50mm</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>标配 120mm 超长高碳钢对穿螺栓</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>空载 190mA，高温 55°C 连续运行峰值堵转 2.4A；强制 500ms 快速热保护</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>SASO (沙特质监认证) / CE EN 12209 Grade 3 / IP65 防尘沙</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>GCC-02</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>gcc-cisa-multipoint</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>euro-cylinder-mortise</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>中东意式多方向防盗联动插芯锁 (Italian Heavy Multipoint Mortise)</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>GCC Italian Style Multi-point Armored Lock</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>阿联酋 / 沙特 / 卡塔尔 (UAE / KSA / Qatar)</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>/assets/img/hero/hero-europe-eurocylinder.jpg</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>/assets/img/hero/hero-europe-eurocylinder.jpg</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>±4.0mm</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>SASO / EN 179 Panic Safe</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>Grade A- (免打孔选配超长紧固件)</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>Yale / Cisa 欧规槽型钥匙</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>BS 85mm 重型深槽，门厚建议 ≥50mm</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>标配 120mm 超长高碳钢对穿螺栓</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>峰值电流 2.8A；配高耐温磷酸铁锂电池与双级硬件过流截断</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>EN 1303 Class 6 / ASTM B117 盐雾 480h / IP65 沙尘</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(taxonomy-8-blocks): deploy 8 industrial divisions 4x2 golden symmetric matrix, restore latin america, and integrate south asia & africa baseline
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/03_GLOBAL_LOCK_DATA_INDEX.xlsx
+++ b/docs/03_GLOBAL_LOCK_DATA_INDEX.xlsx
@@ -788,7 +788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T73"/>
+  <dimension ref="A1:T75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8259,6 +8259,210 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>AF-01</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>af-godrej-rim</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>in-mortise-rim</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>印度与南亚 Godrej 经典三插销外装防撬夜锁 (Godrej Tribolt Rim Deadbolt)</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Godrej Classic Tribolt Rim Deadbolt (India / South Asia)</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>印度 / 南亚 / 东非 (India / South Asia / East Africa)</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>/assets/img/indigenous/uk-nightlatch.jpg</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>/assets/img/indigenous/uk-nightlatch.jpg</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>±3.0mm</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>SASO / EN 179 Panic Safe</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>Grade A- (免打孔选配超长紧固件)</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>Yale / Cisa 欧规槽型钥匙</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>BS 85mm 重型深槽，门厚建议 ≥50mm</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>标配 120mm 超长高碳钢对穿螺栓</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>空载 180mA，堵转峰值 2.0A；配备 500ms 快速过流切断保护</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>BIS (印度国家标准局认证) IS 3818 / 防锯淬火销</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>AF-02</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>af-union-2lever</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>uk-5-lever-mortice</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>非洲南非 Union 经典两拨杆实木门防盗插芯锁 (Union 2-Lever Mortice)</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Union 2-Lever Classic Mortice Lock (South Africa / Nigeria)</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>南非 / 尼日利亚 / 肯尼亚 (South Africa / Nigeria / Kenya)</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>/assets/img/hero/hero-anz-lockwood001.jpg</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>/assets/img/hero/hero-anz-lockwood001.jpg</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>≥ 3.0mm (Door to Frame Gap)</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>≥ 1.2 N·m (Motor torque)</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>±3.5mm</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>SASO / EN 179 Panic Safe</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>Grade A- (免打孔选配超长紧固件)</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>Yale / Cisa 欧规槽型钥匙</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>BS 85mm 重型深槽，门厚建议 ≥50mm</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>标配 120mm 超长高碳钢对穿螺栓</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>空载 200mA，堵转 2.2A</t>
+        </is>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>SABS (南非国家标准局认证) / EN 12209</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>